<commit_message>
SKODA-1001: #485 review: the SK Media Room footer pushed with its newsletter intro
/sk/media-room/footer regenerated with the fixed importer (the intro
beside the nested Subscribe form) and pushed to DA + preview, not
published. Push manifest: that row's new hash; the other 471 rows are
unchanged, back in the tool's key order. Import report updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-locale-footer.report.xlsx
+++ b/tools/importer/reports/import-locale-footer.report.xlsx
@@ -67,7 +67,7 @@
     <t>home-sto</t>
   </si>
   <si>
-    <t>2026-10-28T06:37:06.127Z</t>
+    <t>2026-10-28T06:42:49.315Z</t>
   </si>
   <si>
     <t>Škoda Storyboard</t>
@@ -190,7 +190,7 @@
     <t>images-listing</t>
   </si>
   <si>
-    <t>2026-10-28T06:37:43.635Z</t>
+    <t>2026-10-28T06:43:24.948Z</t>
   </si>
   <si>
     <t>Images - Škoda Storyboard</t>
@@ -232,7 +232,7 @@
     <t>sustainability</t>
   </si>
   <si>
-    <t>2026-10-28T06:38:03.239Z</t>
+    <t>2026-10-28T06:43:42.516Z</t>
   </si>
   <si>
     <t>Sustainable Offices - Škoda Storyboard</t>
@@ -280,7 +280,7 @@
     <t>sk/nav-newsletter</t>
   </si>
   <si>
-    <t>2026-10-28T06:36:56.815Z</t>
+    <t>2026-10-28T06:42:40.559Z</t>
   </si>
   <si>
     <t>https://www.skoda-storyboard.com/sk/</t>
@@ -367,7 +367,7 @@
     <t>sustainability/footer</t>
   </si>
   <si>
-    <t>2026-10-28T06:38:39.618Z</t>
+    <t>2026-10-28T06:44:16.660Z</t>
   </si>
   <si>
     <t>sustainability/nav.report.json</t>
@@ -379,7 +379,7 @@
     <t>sustainability/nav</t>
   </si>
   <si>
-    <t>2026-10-28T06:38:21.162Z</t>
+    <t>2026-10-28T06:43:59.860Z</t>
   </si>
   <si>
     <t>cs/category/e-mobilita-cs.report.json</t>
@@ -598,7 +598,7 @@
     <t>model-page</t>
   </si>
   <si>
-    <t>2026-10-28T06:37:23.860Z</t>
+    <t>2026-10-28T06:43:07.209Z</t>
   </si>
   <si>
     <t>Octavia - Škoda Storyboard</t>
@@ -613,7 +613,7 @@
     <t>sk/media-room/footer</t>
   </si>
   <si>
-    <t>2026-10-27T07:10:33.566Z</t>
+    <t>2026-10-28T09:21:13.160Z</t>
   </si>
   <si>
     <t>https://www.skoda-storyboard.com/sk/media-room/</t>

</xml_diff>